<commit_message>
Fix Orlen LT off-by-one + column parsing, ELVIS DE source, outlier guard, tests, config
</commit_message>
<xml_diff>
--- a/fuel_tracker.xlsx
+++ b/fuel_tracker.xlsx
@@ -12,13 +12,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="+0.000;-0.000;&quot;-&quot;"/>
     <numFmt numFmtId="168" formatCode="+0.0%;-0.0%;&quot;-&quot;"/>
-    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -675,7 +674,7 @@
     </row>
     <row r="5">
       <c r="A5" s="15" t="n">
-        <v>46174.60867165247</v>
+        <v>46174.60867165509</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -692,13 +691,13 @@
         <v>1.5982</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>1.648</v>
+        <v>1.6219</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>-0.0498</v>
+        <v>-0.0237</v>
       </c>
       <c r="H5" s="20" t="n">
-        <v>-0.0302</v>
+        <v>-0.0146</v>
       </c>
       <c r="I5" s="18" t="n">
         <v>1.936</v>
@@ -714,7 +713,7 @@
       </c>
       <c r="M5" s="10" t="inlineStr">
         <is>
-          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl</t>
+          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|LTfix0602</t>
         </is>
       </c>
       <c r="N5" s="11" t="inlineStr">
@@ -742,13 +741,13 @@
         <v>1.6203</v>
       </c>
       <c r="F6" s="18" t="n">
-        <v>1.6731</v>
+        <v>1.648</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>-0.0528</v>
+        <v>-0.0277</v>
       </c>
       <c r="H6" s="20" t="n">
-        <v>-0.0316</v>
+        <v>-0.0168</v>
       </c>
       <c r="I6" s="18" t="n">
         <v>1.936</v>
@@ -764,7 +763,7 @@
       </c>
       <c r="M6" s="10" t="inlineStr">
         <is>
-          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl</t>
+          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|LTfix0602</t>
         </is>
       </c>
       <c r="N6" s="11" t="inlineStr">
@@ -792,13 +791,13 @@
         <v>1.6256</v>
       </c>
       <c r="F7" s="18" t="n">
-        <v>1.7506</v>
+        <v>1.6731</v>
       </c>
       <c r="G7" s="19" t="n">
-        <v>-0.125</v>
+        <v>-0.0475</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>-0.07140000000000001</v>
+        <v>-0.0284</v>
       </c>
       <c r="I7" s="18" t="n">
         <v>1.936</v>
@@ -814,7 +813,7 @@
       </c>
       <c r="M7" s="10" t="inlineStr">
         <is>
-          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|MISS:DE=NO_DATA</t>
+          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|MISS:DE=NO_DATA|LTfix0602</t>
         </is>
       </c>
       <c r="N7" s="11" t="inlineStr">
@@ -842,13 +841,13 @@
         <v>1.6839</v>
       </c>
       <c r="F8" s="18" t="n">
-        <v>1.7623</v>
+        <v>1.7506</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>-0.0784</v>
+        <v>-0.0667</v>
       </c>
       <c r="H8" s="20" t="n">
-        <v>-0.0445</v>
+        <v>-0.0381</v>
       </c>
       <c r="I8" s="18" t="n">
         <v>1.972</v>
@@ -864,7 +863,7 @@
       </c>
       <c r="M8" s="10" t="inlineStr">
         <is>
-          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl</t>
+          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|LTfix0602</t>
         </is>
       </c>
       <c r="N8" s="11" t="inlineStr">
@@ -892,13 +891,13 @@
         <v>1.7252</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>1.768</v>
+        <v>1.7637</v>
       </c>
       <c r="G9" s="19" t="n">
-        <v>-0.0428</v>
+        <v>-0.0385</v>
       </c>
       <c r="H9" s="20" t="n">
-        <v>-0.0242</v>
+        <v>-0.0218</v>
       </c>
       <c r="I9" s="18" t="n">
         <v>1.972</v>
@@ -914,7 +913,7 @@
       </c>
       <c r="M9" s="10" t="inlineStr">
         <is>
-          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl</t>
+          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|LTfix0602</t>
         </is>
       </c>
       <c r="N9" s="11" t="inlineStr">
@@ -942,13 +941,13 @@
         <v>1.7519</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>1.7673</v>
+        <v>1.768</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>-0.0154</v>
+        <v>-0.0161</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>-0.008699999999999999</v>
+        <v>-0.0091</v>
       </c>
       <c r="I10" s="18" t="n">
         <v>1.972</v>
@@ -964,7 +963,7 @@
       </c>
       <c r="M10" s="10" t="inlineStr">
         <is>
-          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl</t>
+          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|LTfix0602</t>
         </is>
       </c>
       <c r="N10" s="11" t="inlineStr">
@@ -992,13 +991,13 @@
         <v>1.7651</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>1.7792</v>
+        <v>1.7673</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>-0.0141</v>
+        <v>-0.0022</v>
       </c>
       <c r="H11" s="20" t="n">
-        <v>-0.007900000000000001</v>
+        <v>-0.0012</v>
       </c>
       <c r="I11" s="18" t="n">
         <v>1.972</v>
@@ -1014,7 +1013,7 @@
       </c>
       <c r="M11" s="10" t="inlineStr">
         <is>
-          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl</t>
+          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|LTfix0602</t>
         </is>
       </c>
       <c r="N11" s="11" t="inlineStr">
@@ -1042,13 +1041,13 @@
         <v>1.7843</v>
       </c>
       <c r="F12" s="18" t="n">
-        <v>1.7916</v>
+        <v>1.7792</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>-0.0073</v>
+        <v>0.0051</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>-0.0041</v>
+        <v>0.0029</v>
       </c>
       <c r="I12" s="18" t="n">
         <v>1.97</v>
@@ -1064,7 +1063,7 @@
       </c>
       <c r="M12" s="10" t="inlineStr">
         <is>
-          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl</t>
+          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|LTfix0602</t>
         </is>
       </c>
       <c r="N12" s="11" t="inlineStr">
@@ -1092,13 +1091,13 @@
         <v>1.793</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>1.7654</v>
+        <v>1.7916</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0.0276</v>
+        <v>0.0014</v>
       </c>
       <c r="H13" s="20" t="n">
-        <v>0.0156</v>
+        <v>0.0008</v>
       </c>
       <c r="I13" s="18" t="n">
         <v>1.97</v>
@@ -1114,7 +1113,7 @@
       </c>
       <c r="M13" s="10" t="inlineStr">
         <is>
-          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl</t>
+          <t>Auto: FX,PL,LT,DE,SE,EU|CLS:Dyzelinas C kl|LTfix0602</t>
         </is>
       </c>
       <c r="N13" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Fix: restore VAT on PL EUR/l (06-15, 06-16); clear bad 0 LT on 06-16
</commit_message>
<xml_diff>
--- a/fuel_tracker.xlsx
+++ b/fuel_tracker.xlsx
@@ -12,13 +12,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="+0.000;-0.000;&quot;-&quot;"/>
-    <numFmt numFmtId="169" formatCode="+0.0%;-0.0%;&quot;-&quot;"/>
+  <numFmts count="5">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="+0.000;-0.000;&quot;-&quot;"/>
+    <numFmt numFmtId="168" formatCode="+0.0%;-0.0%;&quot;-&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -94,9 +93,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -105,19 +104,19 @@
     <xf numFmtId="4" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="166" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -129,9 +128,30 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -651,8 +671,8 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46190.25059968451</v>
+      <c r="A5" s="15" t="n">
+        <v>46190.2505996875</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
@@ -662,25 +682,25 @@
       <c r="C5" s="3" t="n">
         <v>5591</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="16" t="n">
         <v>4.2429</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="17" t="n">
         <v>1.6208</v>
       </c>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="7" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="6" t="n">
+      <c r="F5" s="18" t="n"/>
+      <c r="G5" s="19" t="n"/>
+      <c r="H5" s="20" t="n"/>
+      <c r="I5" s="18" t="n">
         <v>1.7378</v>
       </c>
       <c r="J5" s="9" t="n">
         <v>19.44</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K5" s="16" t="n">
         <v>10.897</v>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="L5" s="17" t="n">
         <v>1.784</v>
       </c>
       <c r="M5" s="10" t="inlineStr">
@@ -712,13 +732,7 @@
         <v>4.246</v>
       </c>
       <c r="E6" t="n">
-        <v>1.334903438530382</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>1.334903438530382</v>
+        <v>1.6419</v>
       </c>
       <c r="I6" t="n">
         <v>1.7547</v>
@@ -756,16 +770,16 @@
         <v>4.246</v>
       </c>
       <c r="E7" t="n">
-        <v>1.318181818181818</v>
+        <v>1.6214</v>
       </c>
       <c r="F7" t="n">
         <v>1.6105</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.2923181818181819</v>
+        <v>0.0109</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.1815077192289239</v>
+        <v>0.0068</v>
       </c>
       <c r="I7" t="n">
         <v>1.765</v>
@@ -5122,31 +5136,31 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="21" t="n">
         <v>46181</v>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B4" s="22" t="n">
         <v>1.8495</v>
       </c>
-      <c r="C4" s="13" t="n">
+      <c r="C4" s="22" t="n">
         <v>1.789</v>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="D4" s="22" t="n">
         <v>1.712</v>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="22" t="n">
         <v>2.1675</v>
       </c>
-      <c r="F4" s="13" t="n">
+      <c r="F4" s="22" t="n">
         <v>1.8471</v>
       </c>
-      <c r="G4" s="13" t="n">
+      <c r="G4" s="22" t="n">
         <v>2.2485</v>
       </c>
-      <c r="H4" s="13" t="n">
+      <c r="H4" s="22" t="n">
         <v>1.8297</v>
       </c>
-      <c r="I4" s="14" t="n">
+      <c r="I4" s="23" t="n">
         <v>0.0108</v>
       </c>
     </row>

</xml_diff>